<commit_message>
Formalize 20260907 draft terms in BuildingComponent
Promote 4 draft terms to enum (batch label 20260907):
- エアシャワー -> MechanicalEquipmentEnum (after 殺菌庫)
- 自動火災報知設備 -> DisasterPreventionEquipmentEnum (after その他防煙設備)
- 洗濯機 -> OtherEquipmentEnum (after 植栽)
- 乾燥機 -> OtherEquipmentEnum (after 洗濯機)

Also update docs/index.html and docs/schemas/index.html:
- Reorder schema list to Japanese-name order
- Change display format to 日本語名（英語名）

Run generate_enum_docs.py, generate_dist.py, generate_enum_excel.py.
Backup: docs/exports/backups/20260920_enum.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/enum.xlsx
+++ b/docs/exports/enum.xlsx
@@ -1254,7 +1254,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>軒天</t>
+          <t>シャッター</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>風除室</t>
+          <t>気密シャッター</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>フロントサッシ</t>
+          <t>軒天</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>自動ドア</t>
+          <t>風除室</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>入口ドア(手動)</t>
+          <t>フロントサッシ</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>開き戸</t>
+          <t>自動ドア</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>引き戸・スライド扉</t>
+          <t>入口ドア(手動)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>窓</t>
+          <t>開き戸</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>トップライト</t>
+          <t>引き戸・スライド扉</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>バルコニー</t>
+          <t>窓</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>雨どい</t>
+          <t>トップライト</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>看板</t>
+          <t>バルコニー</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>煙突</t>
+          <t>雨どい</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>階段</t>
+          <t>看板</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>避難階段</t>
+          <t>煙突</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>その他付属物</t>
+          <t>階段</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1946,12 +1946,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>建物内部</t>
+          <t>建築外部</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>基礎</t>
+          <t>避難階段</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1988,12 +1988,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>建物内部</t>
+          <t>建築外部</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>内壁</t>
+          <t>その他付属物</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>柱</t>
+          <t>基礎</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>誘導設備</t>
+          <t>警報設備</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>梁</t>
+          <t>内壁</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2104,12 +2104,12 @@
     <row r="27">
       <c r="C27" t="inlineStr">
         <is>
-          <t>搬送設備</t>
+          <t>防災設備</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>搬送設備</t>
+          <t>誘導設備</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>天井</t>
+          <t>柱</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2146,12 +2146,12 @@
     <row r="28">
       <c r="C28" t="inlineStr">
         <is>
-          <t>厨房設備</t>
+          <t>搬送設備</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>共用機器</t>
+          <t>搬送設備</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>床</t>
+          <t>梁</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>熱調理機器</t>
+          <t>共用機器</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>廊下</t>
+          <t>天井</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>下調理機</t>
+          <t>熱調理機器</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>階段</t>
+          <t>床</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>冷却と冷凍・冷蔵設備機器</t>
+          <t>下調理機</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>開き戸</t>
+          <t>廊下</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>食器洗浄機・消毒機器</t>
+          <t>冷却と冷凍・冷蔵設備機器</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>引き戸・スライド扉</t>
+          <t>階段</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>サービス機器</t>
+          <t>食器洗浄機・消毒機器</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>踏面</t>
+          <t>開き戸</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>食品廃棄物など処理機器</t>
+          <t>サービス機器</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>蹴上</t>
+          <t>引き戸・スライド扉</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>その他の厨房設備</t>
+          <t>食品廃棄物など処理機器</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>ノンスリップ</t>
+          <t>踏面</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2482,12 +2482,12 @@
     <row r="36">
       <c r="C36" t="inlineStr">
         <is>
-          <t>ガス設備</t>
+          <t>厨房設備</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>配管設備</t>
+          <t>その他の厨房設備</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>カーテンレール</t>
+          <t>蹴上</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>給湯室等設備</t>
+          <t>配管設備</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>ロールスクリーン・ブラインド</t>
+          <t>ノンスリップ</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2566,12 +2566,12 @@
     <row r="38">
       <c r="C38" t="inlineStr">
         <is>
-          <t>観測対象</t>
+          <t>ガス設備</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>観測対象</t>
+          <t>給湯室等設備</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>トイレ</t>
+          <t>カーテンレール</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2608,12 +2608,12 @@
     <row r="39">
       <c r="C39" t="inlineStr">
         <is>
-          <t>その他設備</t>
+          <t>観測対象</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>センサー</t>
+          <t>観測対象</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>浴場・シャワー室</t>
+          <t>ロールスクリーン・ブラインド</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>プール</t>
+          <t>センサー</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>洗い場</t>
+          <t>トイレ</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>水槽</t>
+          <t>プール</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>手摺</t>
+          <t>浴場・シャワー室</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>舞台装置</t>
+          <t>水槽</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>棚</t>
+          <t>洗い場</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2781,17 +2781,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>遊具</t>
+          <t>舞台装置</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>建物外構</t>
+          <t>建物内部</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>フェンス</t>
+          <t>手摺</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2823,17 +2823,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>植栽</t>
+          <t>遊具</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>建物外構</t>
+          <t>建物内部</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>門扉</t>
+          <t>棚</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2865,81 +2865,101 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
+          <t>植栽</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>建物外構</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>フェンス</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>給水機器</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>散水栓</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>厨房用棚類</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>つり棚</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" t="inlineStr">
+        <is>
           <t>その他設備</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>被服関連機器</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
         <is>
           <t>建物外構</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>門扉</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>給水機器</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>弁</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>レンジ</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>オープントップレンジ</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>その他設備</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>その他設備</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>建物外構</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t>コンクリート塀・ブロック塀</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>給水機器</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>散水栓</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>厨房用棚類</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>つり棚</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>建物外構</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>舗装・砂利敷</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>給水機器</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>弁</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>レンジ</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>オープントップレンジ</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>建物外構</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>車止め・縁石・ガードポール</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2971,7 +2991,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>残地・法面</t>
+          <t>舗装・砂利敷</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3003,7 +3023,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>倉庫</t>
+          <t>車止め・縁石・ガードポール</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3035,7 +3055,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>犬走り</t>
+          <t>残地・法面</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3067,7 +3087,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>植栽</t>
+          <t>倉庫</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3099,7 +3119,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>側溝・蓋・枡蓋</t>
+          <t>犬走り</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3131,53 +3151,73 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
+          <t>植栽</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>衛生機器</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>水栓</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>レンジ</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>鋳物コンロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>建物外構</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>側溝・蓋・枡蓋</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>衛生機器</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>自動水栓</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>レンジ</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>電磁調理器</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>建物外構</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
           <t>その他建物外</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>衛生機器</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>水栓</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>レンジ</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>鋳物コンロ</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>衛生機器</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>自動水栓</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>レンジ</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>電磁調理器</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
       <c r="I55" t="inlineStr">
         <is>
           <t>衛生機器</t>
@@ -3427,7 +3467,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>その他衛生器具</t>
+          <t>エアシャワー</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -3444,12 +3484,12 @@
     <row r="67">
       <c r="I67" t="inlineStr">
         <is>
-          <t>給湯機器</t>
+          <t>衛生機器</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>湯沸器</t>
+          <t>その他衛生器具</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -3471,7 +3511,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>ポンプ</t>
+          <t>湯沸器</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -3488,12 +3528,12 @@
     <row r="69">
       <c r="I69" t="inlineStr">
         <is>
-          <t>蒸気設備</t>
+          <t>給湯機器</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>蒸気ボイラー</t>
+          <t>ポンプ</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -3515,7 +3555,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>減圧弁</t>
+          <t>蒸気ボイラー</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -3537,7 +3577,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>安全装置</t>
+          <t>減圧弁</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -3554,12 +3594,12 @@
     <row r="72">
       <c r="I72" t="inlineStr">
         <is>
-          <t>ダクトおよび配管</t>
+          <t>蒸気設備</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>空調ダクト</t>
+          <t>安全装置</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -3581,7 +3621,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>換気ダクト</t>
+          <t>空調ダクト</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -3603,7 +3643,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>給水管</t>
+          <t>換気ダクト</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -3625,7 +3665,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>排水管</t>
+          <t>給水管</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -3647,7 +3687,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>蒸気配管</t>
+          <t>排水管</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -3664,12 +3704,12 @@
     <row r="77">
       <c r="I77" t="inlineStr">
         <is>
-          <t>機能水装置</t>
+          <t>ダクトおよび配管</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>全自動軟水装置</t>
+          <t>蒸気配管</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -3691,7 +3731,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>微酸性水生成器</t>
+          <t>全自動軟水装置</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -3708,12 +3748,12 @@
     <row r="79">
       <c r="I79" t="inlineStr">
         <is>
-          <t>消火設備</t>
+          <t>機能水装置</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>消防設備</t>
+          <t>微酸性水生成器</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -3735,7 +3775,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>ポンプ</t>
+          <t>消防設備</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -3757,7 +3797,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>その他消火設備</t>
+          <t>ポンプ</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -3779,7 +3819,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>防火扉</t>
+          <t>その他消火設備</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -3801,7 +3841,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>防火シャッター</t>
+          <t>防火扉</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -3823,7 +3863,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>防火ダンパー</t>
+          <t>防火シャッター</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -3845,7 +3885,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>防火クロススクリーン</t>
+          <t>防火ダンパー</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -3867,7 +3907,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>ドレンチャー</t>
+          <t>防火クロススクリーン</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -3889,7 +3929,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>その他防火設備</t>
+          <t>ドレンチャー</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -3906,12 +3946,12 @@
     <row r="88">
       <c r="I88" t="inlineStr">
         <is>
-          <t>排煙設備</t>
+          <t>消火設備</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>排煙ファン</t>
+          <t>その他防火設備</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -3933,7 +3973,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>排煙口</t>
+          <t>排煙ファン</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -3955,7 +3995,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>その他排煙設備</t>
+          <t>排煙口</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -3972,12 +4012,12 @@
     <row r="91">
       <c r="I91" t="inlineStr">
         <is>
-          <t>防煙設備</t>
+          <t>排煙設備</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>防煙壁</t>
+          <t>その他排煙設備</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -3999,7 +4039,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>その他防煙設備</t>
+          <t>防煙壁</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -4016,12 +4056,12 @@
     <row r="93">
       <c r="I93" t="inlineStr">
         <is>
-          <t>誘導設備</t>
+          <t>防煙設備</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>非常用照明装置</t>
+          <t>その他防煙設備</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -4038,12 +4078,12 @@
     <row r="94">
       <c r="I94" t="inlineStr">
         <is>
-          <t>誘導設備</t>
+          <t>警報設備</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>誘導灯</t>
+          <t>自動火災報知設備</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -4060,12 +4100,12 @@
     <row r="95">
       <c r="I95" t="inlineStr">
         <is>
-          <t>搬送設備</t>
+          <t>誘導設備</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>コンベア</t>
+          <t>非常用照明装置</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -4082,12 +4122,12 @@
     <row r="96">
       <c r="I96" t="inlineStr">
         <is>
-          <t>搬送設備</t>
+          <t>誘導設備</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>米サイロ</t>
+          <t>誘導灯</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -4109,7 +4149,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>昇降機</t>
+          <t>コンベア</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -4126,12 +4166,12 @@
     <row r="98">
       <c r="I98" t="inlineStr">
         <is>
-          <t>共用機器</t>
+          <t>搬送設備</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>シンク</t>
+          <t>米サイロ</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -4148,12 +4188,12 @@
     <row r="99">
       <c r="I99" t="inlineStr">
         <is>
-          <t>共用機器</t>
+          <t>搬送設備</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>厨房用台類</t>
+          <t>昇降機</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -4175,7 +4215,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>厨房用棚類</t>
+          <t>シンク</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -4192,12 +4232,12 @@
     <row r="101">
       <c r="I101" t="inlineStr">
         <is>
-          <t>熱調理機器</t>
+          <t>共用機器</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>レンジ</t>
+          <t>厨房用台類</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -4214,12 +4254,12 @@
     <row r="102">
       <c r="I102" t="inlineStr">
         <is>
-          <t>熱調理機器</t>
+          <t>共用機器</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>煮炊釜</t>
+          <t>厨房用棚類</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -4241,7 +4281,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>加熱庫</t>
+          <t>レンジ</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -4263,7 +4303,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>焼物器</t>
+          <t>煮炊釜</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -4285,7 +4325,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>揚物器</t>
+          <t>加熱庫</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -4307,7 +4347,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>蒸し器</t>
+          <t>焼物器</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -4329,7 +4369,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>炊飯器</t>
+          <t>揚物器</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -4351,7 +4391,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>その他の熱調理機</t>
+          <t>蒸し器</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -4368,12 +4408,12 @@
     <row r="109">
       <c r="I109" t="inlineStr">
         <is>
-          <t>下調理機</t>
+          <t>熱調理機器</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>食材洗浄機</t>
+          <t>炊飯器</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -4390,12 +4430,12 @@
     <row r="110">
       <c r="I110" t="inlineStr">
         <is>
-          <t>下調理機</t>
+          <t>熱調理機器</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>切裁機</t>
+          <t>その他の熱調理機</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -4417,7 +4457,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>かくはん混合機</t>
+          <t>食材洗浄機</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -4439,7 +4479,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>食品成型機</t>
+          <t>切裁機</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -4461,7 +4501,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>その他の下調理機</t>
+          <t>かくはん混合機</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -4478,12 +4518,12 @@
     <row r="114">
       <c r="I114" t="inlineStr">
         <is>
-          <t>冷却と冷凍・冷蔵設備機器</t>
+          <t>下調理機</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>低温貯蔵保管機器</t>
+          <t>食品成型機</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -4500,12 +4540,12 @@
     <row r="115">
       <c r="I115" t="inlineStr">
         <is>
-          <t>冷却と冷凍・冷蔵設備機器</t>
+          <t>下調理機</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>鮮度向上生産機器</t>
+          <t>その他の下調理機</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -4527,7 +4567,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>低温物流機器</t>
+          <t>低温貯蔵保管機器</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -4549,7 +4589,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>(陳列・展示機器)</t>
+          <t>鮮度向上生産機器</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -4571,7 +4611,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>解凍機器</t>
+          <t>低温物流機器</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -4593,7 +4633,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>製氷機</t>
+          <t>(陳列・展示機器)</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -4615,7 +4655,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>その他の冷却冷凍冷蔵設備</t>
+          <t>解凍機器</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -4632,12 +4672,12 @@
     <row r="121">
       <c r="I121" t="inlineStr">
         <is>
-          <t>食器洗浄機・消毒機器</t>
+          <t>冷却と冷凍・冷蔵設備機器</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>食器洗浄機</t>
+          <t>製氷機</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -4654,12 +4694,12 @@
     <row r="122">
       <c r="I122" t="inlineStr">
         <is>
-          <t>食器洗浄機・消毒機器</t>
+          <t>冷却と冷凍・冷蔵設備機器</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>消毒機器</t>
+          <t>その他の冷却冷凍冷蔵設備</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -4676,12 +4716,12 @@
     <row r="123">
       <c r="I123" t="inlineStr">
         <is>
-          <t>サービス機器</t>
+          <t>食器洗浄機・消毒機器</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>保温機器</t>
+          <t>食器洗浄機</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -4698,12 +4738,12 @@
     <row r="124">
       <c r="I124" t="inlineStr">
         <is>
-          <t>サービス機器</t>
+          <t>食器洗浄機・消毒機器</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>ベーカリー関連機器</t>
+          <t>消毒機器</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -4725,7 +4765,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>配膳車・下膳車</t>
+          <t>保温機器</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -4742,12 +4782,12 @@
     <row r="126">
       <c r="I126" t="inlineStr">
         <is>
-          <t>食品廃棄物など処理機器</t>
+          <t>サービス機器</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>生ごみ処理</t>
+          <t>ベーカリー関連機器</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -4764,12 +4804,12 @@
     <row r="127">
       <c r="I127" t="inlineStr">
         <is>
-          <t>食品廃棄物など処理機器</t>
+          <t>サービス機器</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>コンパクター</t>
+          <t>配膳車・下膳車</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -4791,7 +4831,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>パルパーエストラシステム</t>
+          <t>生ごみ処理</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -4808,12 +4848,12 @@
     <row r="129">
       <c r="I129" t="inlineStr">
         <is>
-          <t>その他の厨房設備</t>
+          <t>食品廃棄物など処理機器</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>金属探知機</t>
+          <t>コンパクター</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -4830,12 +4870,12 @@
     <row r="130">
       <c r="I130" t="inlineStr">
         <is>
-          <t>配管設備</t>
+          <t>食品廃棄物など処理機器</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>ガス栓</t>
+          <t>パルパーエストラシステム</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -4852,12 +4892,12 @@
     <row r="131">
       <c r="I131" t="inlineStr">
         <is>
-          <t>配管設備</t>
+          <t>その他の厨房設備</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>ガス接続具</t>
+          <t>金属探知機</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -4879,7 +4919,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>ガス漏れ警報器等</t>
+          <t>ガス栓</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -4896,12 +4936,12 @@
     <row r="133">
       <c r="I133" t="inlineStr">
         <is>
-          <t>給湯室等設備</t>
+          <t>配管設備</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>ガス器具</t>
+          <t>ガス接続具</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -4918,12 +4958,12 @@
     <row r="134">
       <c r="I134" t="inlineStr">
         <is>
-          <t>観測対象</t>
+          <t>配管設備</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>空間</t>
+          <t>ガス漏れ警報器等</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -4940,12 +4980,12 @@
     <row r="135">
       <c r="I135" t="inlineStr">
         <is>
-          <t>観測対象</t>
+          <t>給湯室等設備</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>ガス器具</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -4967,7 +5007,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>蒸気</t>
+          <t>空間</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -4989,7 +5029,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>(食品)</t>
+          <t>水</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -5006,12 +5046,12 @@
     <row r="138">
       <c r="I138" t="inlineStr">
         <is>
-          <t>センサー</t>
+          <t>観測対象</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>センサー</t>
+          <t>蒸気</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -5028,12 +5068,12 @@
     <row r="139">
       <c r="I139" t="inlineStr">
         <is>
-          <t>センサー</t>
+          <t>観測対象</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>秤</t>
+          <t>(食品)</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -5050,12 +5090,12 @@
     <row r="140">
       <c r="I140" t="inlineStr">
         <is>
-          <t>プール</t>
+          <t>センサー</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>プール</t>
+          <t>センサー</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -5072,12 +5112,12 @@
     <row r="141">
       <c r="I141" t="inlineStr">
         <is>
-          <t>プール</t>
+          <t>センサー</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>プール設備</t>
+          <t>秤</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -5094,12 +5134,12 @@
     <row r="142">
       <c r="I142" t="inlineStr">
         <is>
-          <t>水槽</t>
+          <t>プール</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>水槽</t>
+          <t>プール</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -5116,12 +5156,12 @@
     <row r="143">
       <c r="I143" t="inlineStr">
         <is>
-          <t>舞台装置</t>
+          <t>プール</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>舞台機構</t>
+          <t>プール設備</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -5138,12 +5178,12 @@
     <row r="144">
       <c r="I144" t="inlineStr">
         <is>
-          <t>舞台装置</t>
+          <t>水槽</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>舞台照明</t>
+          <t>水槽</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -5165,7 +5205,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>舞台音響</t>
+          <t>舞台機構</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -5187,7 +5227,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>舞台装置</t>
+          <t>舞台照明</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -5204,12 +5244,12 @@
     <row r="147">
       <c r="I147" t="inlineStr">
         <is>
-          <t>遊具</t>
+          <t>舞台装置</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>遊具</t>
+          <t>舞台音響</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
@@ -5226,12 +5266,12 @@
     <row r="148">
       <c r="I148" t="inlineStr">
         <is>
-          <t>植栽</t>
+          <t>舞台装置</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>植栽</t>
+          <t>舞台装置</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
@@ -5248,12 +5288,12 @@
     <row r="149">
       <c r="I149" t="inlineStr">
         <is>
-          <t>その他設備</t>
+          <t>遊具</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>椅子</t>
+          <t>遊具</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -5270,62 +5310,102 @@
     <row r="150">
       <c r="I150" t="inlineStr">
         <is>
+          <t>植栽</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>植栽</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>配膳車・下膳車</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>冷温蔵配膳車</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>被服関連機器</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>洗濯機</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>配膳車・下膳車</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>常温配膳車</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>被服関連機器</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>乾燥機</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>配膳車・下膳車</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>下膳車</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="I153" t="inlineStr">
+        <is>
           <t>その他設備</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr">
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>椅子</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>生ごみ処理</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>厨芥処理システム</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="I154" t="inlineStr">
         <is>
           <t>その他設備</t>
         </is>
       </c>
-      <c r="L150" t="inlineStr">
-        <is>
-          <t>配膳車・下膳車</t>
-        </is>
-      </c>
-      <c r="M150" t="inlineStr">
-        <is>
-          <t>冷温蔵配膳車</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>配膳車・下膳車</t>
-        </is>
-      </c>
-      <c r="M151" t="inlineStr">
-        <is>
-          <t>常温配膳車</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>配膳車・下膳車</t>
-        </is>
-      </c>
-      <c r="M152" t="inlineStr">
-        <is>
-          <t>下膳車</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>生ごみ処理</t>
-        </is>
-      </c>
-      <c r="M153" t="inlineStr">
-        <is>
-          <t>厨芥処理システム</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>その他設備</t>
+        </is>
+      </c>
       <c r="L154" t="inlineStr">
         <is>
           <t>生ごみ処理</t>

</xml_diff>